<commit_message>
feat(carnegie): connect MTC as an illustrative research candidate
Add a distinct organization record, three reviewed sources, and a small workbook/demo example. Keep the NYIMF/Troen match unconfirmed and the partner sheet separate. Preserve school records and edited exports; retain source-review corrections and aggregate page accounting. Verified with 15 focused tests, workbook reconciliation, and desktop/mobile viewport review.

Co-Authored-By: Codex <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/demo/carnegie-hall/outputs/01a08da2-45ab-7181-a80f-a887cb079101/Troen - Carnegie Opportunity Review.xlsx
+++ b/demo/carnegie-hall/outputs/01a08da2-45ab-7181-a80f-a887cb079101/Troen - Carnegie Opportunity Review.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Opportunities" sheetId="1" r:id="Rde83c261d64540bf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence" sheetId="2" r:id="R70a147b7c5f04c63"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Opportunities" sheetId="1" r:id="R230cfd2777724d7c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence" sheetId="2" r:id="R57aff047074248b1"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -167,10 +167,10 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="OpportunityReview" displayName="OpportunityReview" ref="A6:F8" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A6:F8"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="OpportunityReview" displayName="OpportunityReview" ref="A6:F9" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A6:F9"/>
   <x:tableColumns count="6">
-    <x:tableColumn id="1" name="School / location"/>
+    <x:tableColumn id="1" name="Organization / location"/>
     <x:tableColumn id="2" name="Research interpretation"/>
     <x:tableColumn id="3" name="Next internal step"/>
     <x:tableColumn id="4" name="Disposition"/>
@@ -182,11 +182,11 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="PublicEvidence" displayName="PublicEvidence" ref="A6:G15" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A6:G15"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="PublicEvidence" displayName="PublicEvidence" ref="A6:G18" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A6:G18"/>
   <x:tableColumns count="7">
     <x:tableColumn id="1" name="Source ID"/>
-    <x:tableColumn id="2" name="School record"/>
+    <x:tableColumn id="2" name="Organization record"/>
     <x:tableColumn id="3" name="Observed fact / source context"/>
     <x:tableColumn id="4" name="Evidence date or period"/>
     <x:tableColumn id="5" name="Checked"/>
@@ -423,7 +423,7 @@
     </x:row>
     <x:row r="3" ht="23" customHeight="1">
       <x:c r="A3" s="2" t="str">
-        <x:v>March 3, 2027 • 2 research examples; interest, availability and eligibility are unverified.</x:v>
+        <x:v>March 3, 2027 • 3 research examples; interest, availability and eligibility are unverified.</x:v>
       </x:c>
       <x:c r="B3" s="2"/>
       <x:c r="C3" s="2"/>
@@ -451,7 +451,7 @@
     </x:row>
     <x:row r="6" ht="32" customHeight="1">
       <x:c r="A6" s="13" t="str">
-        <x:v>School / location</x:v>
+        <x:v>Organization / location</x:v>
       </x:c>
       <x:c r="B6" s="14" t="str">
         <x:v>Research interpretation</x:v>
@@ -507,26 +507,46 @@
         <x:v>salem-concert-band-carnegie-2027-03-03</x:v>
       </x:c>
     </x:row>
-    <x:row r="9">
-      <x:c r="A9" s="2"/>
-      <x:c r="B9" s="2"/>
-      <x:c r="C9" s="2"/>
-      <x:c r="D9" s="2"/>
-      <x:c r="E9" s="2"/>
-      <x:c r="F9" s="2"/>
+    <x:row r="9" ht="92" customHeight="1">
+      <x:c r="A9" s="8" t="str">
+        <x:v>Music Travel Consultants (MTC)
+Indianapolis, IN
+Candidate: Student music tour operator</x:v>
+      </x:c>
+      <x:c r="B9" s="8" t="str">
+        <x:v>MTC markets music travel and lists a planned March 3 NYIMF event. The NYIMF/Troen match is unconfirmed. This is an illustrative research candidate.</x:v>
+      </x:c>
+      <x:c r="C9" s="8" t="str">
+        <x:v>Research example only. Troen relationship and interest are unknown. No recommendation to contact MTC.</x:v>
+      </x:c>
+      <x:c r="D9" s="16" t="str">
+        <x:v>To review</x:v>
+      </x:c>
+      <x:c r="E9" s="16"/>
+      <x:c r="F9" s="8" t="str">
+        <x:v>mtc-research-carnegie-2027-03-03</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="2"/>
+      <x:c r="B10" s="2"/>
+      <x:c r="C10" s="2"/>
+      <x:c r="D10" s="2"/>
+      <x:c r="E10" s="2"/>
+      <x:c r="F10" s="2"/>
     </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="D7:D8">
+  <x:conditionalFormatting sqref="D7:D9">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="Park"/>
   </x:conditionalFormatting>
   <x:dataValidations count="1">
-    <x:dataValidation type="list" sqref="D7:D8">
+    <x:dataValidation type="list" sqref="D7:D9">
       <x:formula1>"To review,Keep researching,Park"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R58b81c265a6b4fa0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6d7ec0f3eee4403d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -600,7 +620,7 @@
         <x:v>Source ID</x:v>
       </x:c>
       <x:c r="B6" s="14" t="str">
-        <x:v>School record</x:v>
+        <x:v>Organization record</x:v>
       </x:c>
       <x:c r="C6" s="14" t="str">
         <x:v>Observed fact / source context</x:v>
@@ -834,10 +854,82 @@
         <x:v>https://salemmarchingband.wixsite.com/home</x:v>
       </x:c>
     </x:row>
+    <x:row r="16" ht="78" customHeight="1">
+      <x:c r="A16" s="8" t="str">
+        <x:v>MTC-02</x:v>
+      </x:c>
+      <x:c r="B16" s="8" t="str">
+        <x:v>Music Travel Consultants (MTC)
+Indianapolis, IN</x:v>
+      </x:c>
+      <x:c r="C16" s="8" t="str">
+        <x:v>MTC describes itself as an Indianapolis-based tour operator creating customized trips for student music groups. Company self-description; undated. Pilot claim C1.</x:v>
+      </x:c>
+      <x:c r="D16" s="17" t="str">
+        <x:v>Undated page</x:v>
+      </x:c>
+      <x:c r="E16" s="17" t="n">
+        <x:v>46276</x:v>
+      </x:c>
+      <x:c r="F16" s="8" t="str">
+        <x:v>Company website</x:v>
+      </x:c>
+      <x:c r="G16" s="18" t="str">
+        <x:v>https://www.musictravel.com/about.html</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="78" customHeight="1">
+      <x:c r="A17" s="8" t="str">
+        <x:v>MTC-01</x:v>
+      </x:c>
+      <x:c r="B17" s="8" t="str">
+        <x:v>Music Travel Consultants (MTC)
+Indianapolis, IN</x:v>
+      </x:c>
+      <x:c r="C17" s="8" t="str">
+        <x:v>Its New York City page includes Carnegie Hall among performance-travel options. Marketing copy does not establish a completed MTC trip. Service description, not dated performance evidence. Pilot claim C6.</x:v>
+      </x:c>
+      <x:c r="D17" s="17" t="str">
+        <x:v>Undated page</x:v>
+      </x:c>
+      <x:c r="E17" s="17" t="n">
+        <x:v>46276</x:v>
+      </x:c>
+      <x:c r="F17" s="8" t="str">
+        <x:v>Company marketing</x:v>
+      </x:c>
+      <x:c r="G17" s="18" t="str">
+        <x:v>https://www.musictravel.com/new-york-city/new-york-city-performance-trips.html</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="78" customHeight="1">
+      <x:c r="A18" s="8" t="str">
+        <x:v>MTC-05</x:v>
+      </x:c>
+      <x:c r="B18" s="8" t="str">
+        <x:v>Music Travel Consultants (MTC)
+Indianapolis, IN</x:v>
+      </x:c>
+      <x:c r="C18" s="8" t="str">
+        <x:v>Its 2027 calendar lists the New York Invitational Music Festival at Carnegie Hall on March 3 for high school bands, choirs and orchestras. No reviewed page names Troen as producer. Published March 17, 2026; updated April 20. Also lists March 31, outside this POC. NYIMF/Troen match unconfirmed. Pilot C7/U1.</x:v>
+      </x:c>
+      <x:c r="D18" s="17" t="str">
+        <x:v>Planned: March 3, 2027</x:v>
+      </x:c>
+      <x:c r="E18" s="17" t="n">
+        <x:v>46276</x:v>
+      </x:c>
+      <x:c r="F18" s="8" t="str">
+        <x:v>Planned event listing</x:v>
+      </x:c>
+      <x:c r="G18" s="18" t="str">
+        <x:v>https://www.musictravel.com/blog/2026/03/17/the-carnegie-hall-experience-2027-student-music-festivals/</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra2a5dac2abd443c0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4f2e1f6df70b4787"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>